<commit_message>
Sanitize public QC terminology
</commit_message>
<xml_diff>
--- a/supporting_information/S3_Transferability_Supplement.xlsx
+++ b/supporting_information/S3_Transferability_Supplement.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25_summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S26_TCGA_precomputed" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S27_manifest" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S28_review" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S28_quality_checks" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -564,12 +564,12 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>executor_agent_id</t>
+          <t>analysis_role_id</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_agent_id</t>
+          <t>qc_role_id</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>0.209691</t>
@@ -677,12 +676,12 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -767,7 +766,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>0.209691</t>
@@ -790,12 +788,12 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -880,7 +878,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>-0.0496982</t>
@@ -903,12 +900,12 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -993,7 +990,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>-0.0496982</t>
@@ -1016,12 +1012,12 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1102,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>0.110698</t>
@@ -1129,12 +1124,12 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1214,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>0.110698</t>
@@ -1242,12 +1236,12 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1326,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>-0.422435</t>
@@ -1355,12 +1348,12 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1438,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
           <t>-0.422435</t>
@@ -1468,12 +1460,12 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1550,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>-0.278605</t>
@@ -1581,12 +1572,12 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1662,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>-0.278605</t>
@@ -1694,12 +1684,12 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1774,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>-0.317807</t>
@@ -1807,12 +1796,12 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1886,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>-0.317807</t>
@@ -1920,12 +1908,12 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2010,7 +1998,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>0.24393</t>
@@ -2033,12 +2020,12 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2110,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>0.24393</t>
@@ -2146,12 +2132,12 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2222,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>0.395708</t>
@@ -2259,12 +2244,12 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2334,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>0.395708</t>
@@ -2372,12 +2356,12 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2446,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>-0.144098</t>
@@ -2485,12 +2468,12 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2558,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>-0.144098</t>
@@ -2598,12 +2580,12 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2670,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>0.674145</t>
@@ -2711,12 +2692,12 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2782,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>0.674145</t>
@@ -2824,12 +2804,12 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2894,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>0.116398</t>
@@ -2937,12 +2916,12 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3006,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>0.116398</t>
@@ -3050,12 +3028,12 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3118,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>0.199899</t>
@@ -3163,12 +3140,12 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3230,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>0.199899</t>
@@ -3276,12 +3252,12 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3342,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>0.0509054</t>
@@ -3389,12 +3364,12 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3454,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>0.0509054</t>
@@ -3502,12 +3476,12 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3566,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
           <t>-0.00288397</t>
@@ -3615,12 +3588,12 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3678,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
           <t>-0.00288397</t>
@@ -3728,12 +3700,12 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3790,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
           <t>0.116365</t>
@@ -3841,12 +3812,12 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3902,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
           <t>0.116365</t>
@@ -3954,12 +3924,12 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4014,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>-0.0396043</t>
@@ -4067,12 +4036,12 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4126,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>-0.0396043</t>
@@ -4180,12 +4148,12 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4238,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
           <t>0.184272</t>
@@ -4293,12 +4260,12 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4350,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>0.184272</t>
@@ -4406,12 +4372,12 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4462,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
           <t>-0.38786</t>
@@ -4519,12 +4484,12 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4574,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>-0.38786</t>
@@ -4632,12 +4596,12 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4686,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
           <t>-0.265258</t>
@@ -4745,12 +4708,12 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4798,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>-0.265258</t>
@@ -4858,12 +4820,12 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -4948,7 +4910,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
           <t>-0.300235</t>
@@ -4971,12 +4932,12 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5022,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>-0.300235</t>
@@ -5084,12 +5044,12 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5134,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>0.171999</t>
@@ -5197,12 +5156,12 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5246,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>0.171999</t>
@@ -5310,12 +5268,12 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5358,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>0.376559</t>
@@ -5423,12 +5380,12 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5513,7 +5470,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>0.376559</t>
@@ -5536,12 +5492,12 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5582,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>-0.113749</t>
@@ -5649,12 +5604,12 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5739,7 +5694,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
           <t>-0.113749</t>
@@ -5762,12 +5716,12 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5806,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
           <t>0.638464</t>
@@ -5875,12 +5828,12 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5918,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
           <t>0.638464</t>
@@ -5988,12 +5940,12 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6078,7 +6030,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
           <t>0.168176</t>
@@ -6101,12 +6052,12 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6142,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
           <t>0.168176</t>
@@ -6214,12 +6164,12 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6254,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
           <t>0.225721</t>
@@ -6327,12 +6276,12 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6417,7 +6366,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
           <t>0.225721</t>
@@ -6440,12 +6388,12 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6530,7 +6478,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
           <t>0.0459759</t>
@@ -6553,12 +6500,12 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6643,7 +6590,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
           <t>0.0459759</t>
@@ -6666,12 +6612,12 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6702,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
           <t>0.0321596</t>
@@ -6779,12 +6724,12 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6814,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
           <t>0.0321596</t>
@@ -6892,12 +6836,12 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7006,12 +6950,12 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>executor_agent_id</t>
+          <t>analysis_role_id</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_agent_id</t>
+          <t>qc_role_id</t>
         </is>
       </c>
     </row>
@@ -7088,12 +7032,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7170,12 +7114,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7252,12 +7196,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7334,12 +7278,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7416,12 +7360,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7498,12 +7442,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7580,12 +7524,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7662,12 +7606,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7758,12 +7702,12 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>executor_agent_id</t>
+          <t>analysis_role_id</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_agent_id</t>
+          <t>qc_role_id</t>
         </is>
       </c>
     </row>
@@ -7825,12 +7769,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7892,12 +7836,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7959,12 +7903,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8026,12 +7970,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8093,12 +8037,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8160,12 +8104,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8227,12 +8171,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8294,12 +8238,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8361,12 +8305,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8428,12 +8372,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8495,12 +8439,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8562,12 +8506,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8629,12 +8573,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8696,12 +8640,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8763,12 +8707,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8830,12 +8774,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8897,12 +8841,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -8964,12 +8908,12 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9031,12 +8975,12 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9098,12 +9042,12 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9165,12 +9109,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9232,12 +9176,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9299,12 +9243,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9366,12 +9310,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9433,12 +9377,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9500,12 +9444,12 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9567,12 +9511,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9634,12 +9578,12 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9701,12 +9645,12 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9768,12 +9712,12 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9835,12 +9779,12 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9902,12 +9846,12 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -9969,12 +9913,12 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10036,12 +9980,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10103,12 +10047,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10170,12 +10114,12 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10237,12 +10181,12 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10352,17 +10296,17 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>claim_boundary</t>
+          <t>interpretation_scope</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>executor_agent_id</t>
+          <t>analysis_role_id</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_agent_id</t>
+          <t>qc_role_id</t>
         </is>
       </c>
     </row>
@@ -10444,12 +10388,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10531,12 +10475,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10639,12 +10583,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>executor_agent_id</t>
+          <t>analysis_role_id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_agent_id</t>
+          <t>qc_role_id</t>
         </is>
       </c>
     </row>
@@ -10674,8 +10618,6 @@
           <t>653</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>-2.4928</t>
@@ -10691,8 +10633,6 @@
           <t>0.82513</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>precomputed public bulk layer reused from earlier successful workflow run</t>
@@ -10700,12 +10640,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10735,8 +10675,6 @@
           <t>653</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>2.61812</t>
@@ -10752,8 +10690,6 @@
           <t>8.61082e-40</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>precomputed public bulk layer reused from earlier successful workflow run</t>
@@ -10761,12 +10697,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10791,7 +10727,6 @@
           <t>92</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>92</t>
@@ -10802,9 +10737,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>0.644208</t>
@@ -10822,12 +10754,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10852,7 +10784,6 @@
           <t>92</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>92</t>
@@ -10863,9 +10794,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>0.449715</t>
@@ -10883,12 +10811,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10967,7 +10895,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>URLError: &lt;urlopen error [SSL: UNEXPECTED_EOF_WHILE_READING] EOF occurred in violation of protocol (_ssl.c:1010)&gt;</t>
@@ -11000,7 +10927,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11042,29 +10968,29 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_comment</t>
+          <t>qc_comment</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>executor_agent_id</t>
+          <t>analysis_role_id</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>reviewer_agent_id</t>
+          <t>qc_role_id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>agent_separation</t>
+          <t>role_separation</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>executor_reviewer_distinct</t>
+          <t>independent_qc_roles</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -11074,17 +11000,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Executor and reviewer IDs are distinct.</t>
+          <t>Analysis and QC role IDs are distinct.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -11111,12 +11037,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -11143,19 +11069,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>claim_boundary</t>
+          <t>interpretation_scope</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -11175,12 +11101,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>transferability_executor_001</t>
+          <t>transferability_analysis_001</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>transferability_reviewer_001</t>
+          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prepare v1.0.10 consistency release
</commit_message>
<xml_diff>
--- a/supporting_information/S3_Transferability_Supplement.xlsx
+++ b/supporting_information/S3_Transferability_Supplement.xlsx
@@ -13,7 +13,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25_summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S26_TCGA_precomputed" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S27_manifest" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S28_quality_checks" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W57"/>
+  <dimension ref="A1:U57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -562,16 +561,6 @@
           <t>comparison_expectation</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>analysis_batch_id</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>quality_check_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -674,16 +663,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -786,16 +765,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -898,16 +867,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1010,16 +969,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1122,16 +1071,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1234,16 +1173,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1346,16 +1275,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1458,16 +1377,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1570,16 +1479,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1682,16 +1581,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1794,16 +1683,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1906,16 +1785,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2018,16 +1887,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2130,16 +1989,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2242,16 +2091,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2354,16 +2193,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2466,16 +2295,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2578,16 +2397,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2690,16 +2499,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2802,16 +2601,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2914,16 +2703,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3026,16 +2805,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3138,16 +2907,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3250,16 +3009,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3362,16 +3111,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3474,16 +3213,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3586,16 +3315,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3698,16 +3417,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W29" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3810,16 +3519,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3922,16 +3621,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4034,16 +3723,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4146,16 +3825,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4258,16 +3927,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4370,16 +4029,6 @@
           <t>expected_inverse_or_weak</t>
         </is>
       </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W35" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4482,16 +4131,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4594,16 +4233,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W37" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4706,16 +4335,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4818,16 +4437,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4930,16 +4539,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W40" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5042,16 +4641,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W41" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5154,16 +4743,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W42" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5266,16 +4845,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W43" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5378,16 +4947,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W44" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5490,16 +5049,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W45" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5602,16 +5151,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W46" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5714,16 +5253,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W47" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5826,16 +5355,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W48" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5938,16 +5457,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W49" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6050,16 +5559,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6162,16 +5661,6 @@
           <t>expected_positive_or_contextual</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6274,16 +5763,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6386,16 +5865,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6498,16 +5967,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V54" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W54" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6610,16 +6069,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V55" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W55" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6722,16 +6171,6 @@
           <t>contextual</t>
         </is>
       </c>
-      <c r="V56" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W56" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6832,16 +6271,6 @@
       <c r="U57" t="inlineStr">
         <is>
           <t>contextual</t>
-        </is>
-      </c>
-      <c r="V57" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="W57" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6948,16 +6377,6 @@
           <t>interpretation</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>analysis_batch_id</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>quality_check_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7030,16 +6449,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7112,16 +6521,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7194,16 +6593,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7276,16 +6665,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7358,16 +6737,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7440,16 +6809,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7522,16 +6881,6 @@
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7602,16 +6951,6 @@
       <c r="N9" t="inlineStr">
         <is>
           <t>source-table ROI-level progression quantification; not direct CAF-JAG1-NOTCH1 ligand-receptor evidence</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -7626,7 +6965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7700,16 +7039,6 @@
           <t>interpretation</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>analysis_batch_id</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>quality_check_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7767,16 +7096,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7834,16 +7153,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7901,16 +7210,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7968,16 +7267,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8035,16 +7324,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8102,16 +7381,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8169,16 +7438,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8236,16 +7495,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8303,16 +7552,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8370,16 +7609,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8437,16 +7666,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8504,16 +7723,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8571,16 +7780,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8638,16 +7837,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8705,16 +7894,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8772,16 +7951,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8839,16 +8008,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8906,16 +8065,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8973,16 +8122,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9040,16 +8179,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9107,16 +8236,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9174,16 +8293,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9241,16 +8350,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9308,16 +8407,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9375,16 +8464,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9442,16 +8521,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9509,16 +8578,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9576,16 +8635,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9643,16 +8692,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9710,16 +8749,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9777,16 +8806,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9844,16 +8863,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9911,16 +8920,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9978,16 +8977,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10045,16 +9034,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10112,16 +9091,6 @@
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10177,16 +9146,6 @@
       <c r="K38" t="inlineStr">
         <is>
           <t>supportive source-table row for transferability phenotype; not raw spatial reanalysis</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10201,7 +9160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10291,22 +9250,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>transferability_status</t>
+          <t>transferability_assessment</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>interpretation_scope</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>analysis_batch_id</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -10378,22 +9327,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>supports framework transferability at association/source-table level only; not a new mechanism or clinical biomarker</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10465,22 +9404,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
           <t>supports framework transferability at association/source-table level only; not a new mechanism or clinical biomarker</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10495,7 +9424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10581,16 +9510,6 @@
           <t>interpretation</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>analysis_batch_id</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>quality_check_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10638,16 +9557,6 @@
           <t>precomputed public bulk layer reused from earlier successful workflow run</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10695,16 +9604,6 @@
           <t>precomputed public bulk layer reused from earlier successful workflow run</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10752,16 +9651,6 @@
           <t>precomputed public bulk survival layer reused; no prognostic claim unless supported</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10807,16 +9696,6 @@
       <c r="M5" t="inlineStr">
         <is>
           <t>precomputed public bulk survival layer reused; no prognostic claim unless supported</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>
@@ -10882,7 +9761,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>failed</t>
+          <t>not_used_for_transferability_supplement</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10897,7 +9776,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>URLError: &lt;urlopen error [SSL: UNEXPECTED_EOF_WHILE_READING] EOF occurred in violation of protocol (_ssl.c:1010)&gt;</t>
+          <t>TCGA transferability evidence was read from precomputed submitted tables; no additional Xena download was required for this supplement.</t>
         </is>
       </c>
     </row>
@@ -10925,188 +9804,6 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>69</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>stage</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>qc_comment</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>analysis_batch_id</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>quality_check_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>quality_check_structure</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>independent_qc_roles</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>pass</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Analysis and QC role IDs are distinct.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>bulk_validation</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>tcga_or_geo_completed</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>pass_with_limits</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>At least one public bulk layer loaded; interpret as association-level evidence.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>source_table_reproducibility</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>hra003627_stage_trend_present</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>pass_with_limits</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>HRA003627 source-table trends support transferability demonstration; source tables are not raw spatial matrices.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>interpretation_scope</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>no_new_mechanistic_or_clinical_claim</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>pass</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Use only as supplemental framework portability evidence.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>transferability_analysis_001</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>transferability_qc_001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prepare v1.0.12 final submission package
</commit_message>
<xml_diff>
--- a/supporting_information/S3_Transferability_Supplement.xlsx
+++ b/supporting_information/S3_Transferability_Supplement.xlsx
@@ -9554,7 +9554,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>precomputed public bulk layer reused from earlier successful workflow run</t>
+          <t>precomputed public bulk layer reused from same public-data workflow</t>
         </is>
       </c>
     </row>
@@ -9601,7 +9601,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>precomputed public bulk layer reused from earlier successful workflow run</t>
+          <t>precomputed public bulk layer reused from same public-data workflow</t>
         </is>
       </c>
     </row>

</xml_diff>